<commit_message>
feat(calculators): first test case for 16.5 passing
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/16-lulucf/16.1-lulucf.xlsx
+++ b/packages/calculators/src/modules/test/16-lulucf/16.1-lulucf.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/16-lulucf/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{083C44B4-6804-0648-9E18-AA86D87208C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{467B2523-29EF-0742-9B74-29AC65CA6F22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51200" yWindow="13240" windowWidth="28800" windowHeight="27420" activeTab="2" xr2:uid="{CC0FEAF9-C40F-694B-BCB9-117AFB86C05D}"/>
+    <workbookView xWindow="51200" yWindow="13240" windowWidth="28800" windowHeight="27420" activeTab="3" xr2:uid="{CC0FEAF9-C40F-694B-BCB9-117AFB86C05D}"/>
   </bookViews>
   <sheets>
     <sheet name="16.1.1.2" sheetId="1" r:id="rId1"/>
@@ -983,7 +983,8 @@
         <v>23</v>
       </c>
       <c r="P7">
-        <v>3.67</v>
+        <f>44/12</f>
+        <v>3.6666666666666665</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
@@ -1106,11 +1107,11 @@
       </c>
       <c r="J11">
         <f>$P$7</f>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="K11">
         <f>I11*J11*-1</f>
-        <v>-183.5</v>
+        <v>-183.33333333333331</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
@@ -1146,11 +1147,11 @@
       </c>
       <c r="J12">
         <f>$P$7</f>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="K12">
         <f>I12*J12*-1</f>
-        <v>7156.5</v>
+        <v>7150</v>
       </c>
     </row>
   </sheetData>
@@ -1295,7 +1296,8 @@
         <v>23</v>
       </c>
       <c r="M7">
-        <v>3.67</v>
+        <f>44/12</f>
+        <v>3.6666666666666665</v>
       </c>
     </row>
     <row r="9" spans="1:13" s="1" customFormat="1" ht="51" x14ac:dyDescent="0.2">
@@ -1349,11 +1351,11 @@
       </c>
       <c r="E11">
         <f>$M$7</f>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F11">
         <f>D11*E11*-1</f>
-        <v>0.44039999999999996</v>
+        <v>0.43999999999999995</v>
       </c>
       <c r="K11" s="7" t="s">
         <v>50</v>
@@ -1379,11 +1381,11 @@
       </c>
       <c r="E12">
         <f t="shared" ref="E12:E75" si="2">$M$7</f>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F12">
         <f t="shared" ref="F12:F75" si="3">D12*E12*-1</f>
-        <v>2.8626</v>
+        <v>2.86</v>
       </c>
       <c r="K12" s="7" t="s">
         <v>51</v>
@@ -1409,11 +1411,11 @@
       </c>
       <c r="E13">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F13">
         <f t="shared" si="3"/>
-        <v>0.9909</v>
+        <v>0.99</v>
       </c>
       <c r="K13" s="7" t="s">
         <v>52</v>
@@ -1439,11 +1441,11 @@
       </c>
       <c r="E14">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F14">
         <f t="shared" si="3"/>
-        <v>1.3211999999999999</v>
+        <v>1.3199999999999998</v>
       </c>
       <c r="K14" s="7" t="s">
         <v>53</v>
@@ -1469,11 +1471,11 @@
       </c>
       <c r="E15">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F15">
         <f t="shared" si="3"/>
-        <v>2.3855</v>
+        <v>2.3833333333333333</v>
       </c>
       <c r="K15" s="7" t="s">
         <v>54</v>
@@ -1499,11 +1501,11 @@
       </c>
       <c r="E16">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F16">
         <f t="shared" si="3"/>
-        <v>2.8626</v>
+        <v>2.86</v>
       </c>
       <c r="K16" s="7" t="s">
         <v>55</v>
@@ -1529,11 +1531,11 @@
       </c>
       <c r="E17">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F17">
         <f t="shared" si="3"/>
-        <v>14.129500000000002</v>
+        <v>14.116666666666669</v>
       </c>
       <c r="K17" s="7" t="s">
         <v>56</v>
@@ -1559,11 +1561,11 @@
       </c>
       <c r="E18">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F18">
         <f t="shared" si="3"/>
-        <v>0.29360000000000003</v>
+        <v>0.29333333333333333</v>
       </c>
       <c r="K18" s="7" t="s">
         <v>57</v>
@@ -1589,11 +1591,11 @@
       </c>
       <c r="E19">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F19">
         <f t="shared" si="3"/>
-        <v>2.3121000000000005</v>
+        <v>2.3100000000000005</v>
       </c>
       <c r="K19" s="7" t="s">
         <v>58</v>
@@ -1619,11 +1621,11 @@
       </c>
       <c r="E20">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F20">
         <f t="shared" si="3"/>
-        <v>2.202</v>
+        <v>2.1999999999999997</v>
       </c>
       <c r="K20" s="7" t="s">
         <v>59</v>
@@ -1649,11 +1651,11 @@
       </c>
       <c r="E21">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F21">
         <f t="shared" si="3"/>
-        <v>3.6332999999999998</v>
+        <v>3.63</v>
       </c>
       <c r="K21" s="7" t="s">
         <v>60</v>
@@ -1679,11 +1681,11 @@
       </c>
       <c r="E22">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F22">
         <f t="shared" si="3"/>
-        <v>8.3676000000000013</v>
+        <v>8.3600000000000012</v>
       </c>
       <c r="K22" s="7" t="s">
         <v>61</v>
@@ -1709,11 +1711,11 @@
       </c>
       <c r="E23">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F23">
         <f t="shared" si="3"/>
-        <v>6.2022999999999993</v>
+        <v>6.1966666666666663</v>
       </c>
       <c r="K23" s="7" t="s">
         <v>62</v>
@@ -1739,11 +1741,11 @@
       </c>
       <c r="E24">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F24">
         <f t="shared" si="3"/>
-        <v>2.0552000000000001</v>
+        <v>2.0533333333333332</v>
       </c>
       <c r="K24" s="7" t="s">
         <v>63</v>
@@ -1769,11 +1771,11 @@
       </c>
       <c r="E25">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F25">
         <f t="shared" si="3"/>
-        <v>22.02</v>
+        <v>22</v>
       </c>
       <c r="K25" s="7" t="s">
         <v>64</v>
@@ -1799,11 +1801,11 @@
       </c>
       <c r="E26">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F26">
         <f t="shared" si="3"/>
-        <v>5.2847999999999997</v>
+        <v>5.2799999999999994</v>
       </c>
       <c r="K26" s="7" t="s">
         <v>65</v>
@@ -1829,7 +1831,7 @@
       </c>
       <c r="E27">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F27">
         <f t="shared" si="3"/>
@@ -1859,11 +1861,11 @@
       </c>
       <c r="E28">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F28">
         <f t="shared" si="3"/>
-        <v>29.066399999999998</v>
+        <v>29.04</v>
       </c>
       <c r="K28" s="7" t="s">
         <v>67</v>
@@ -1889,11 +1891,11 @@
       </c>
       <c r="E29">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F29">
         <f t="shared" si="3"/>
-        <v>14.643299999999998</v>
+        <v>14.629999999999999</v>
       </c>
       <c r="K29" s="7" t="s">
         <v>68</v>
@@ -1919,11 +1921,11 @@
       </c>
       <c r="E30">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F30">
         <f t="shared" si="3"/>
-        <v>15.414</v>
+        <v>15.4</v>
       </c>
       <c r="K30" s="7" t="s">
         <v>69</v>
@@ -1949,7 +1951,7 @@
       </c>
       <c r="E31">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F31">
         <f t="shared" si="3"/>
@@ -1979,11 +1981,11 @@
       </c>
       <c r="E32">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F32">
         <f t="shared" si="3"/>
-        <v>3.2296</v>
+        <v>3.2266666666666666</v>
       </c>
       <c r="K32" s="7" t="s">
         <v>71</v>
@@ -2009,11 +2011,11 @@
       </c>
       <c r="E33">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F33">
         <f t="shared" si="3"/>
-        <v>5.9087000000000005</v>
+        <v>5.9033333333333333</v>
       </c>
       <c r="K33" s="7" t="s">
         <v>72</v>
@@ -2039,11 +2041,11 @@
       </c>
       <c r="E34">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F34">
         <f t="shared" si="3"/>
-        <v>3.5231999999999997</v>
+        <v>3.5199999999999996</v>
       </c>
       <c r="K34" s="7" t="s">
         <v>73</v>
@@ -2069,11 +2071,11 @@
       </c>
       <c r="E35">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F35">
         <f t="shared" si="3"/>
-        <v>22.02</v>
+        <v>22</v>
       </c>
       <c r="K35" s="7" t="s">
         <v>74</v>
@@ -2099,11 +2101,11 @@
       </c>
       <c r="E36">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F36">
         <f t="shared" si="3"/>
-        <v>16.221399999999999</v>
+        <v>16.206666666666667</v>
       </c>
       <c r="K36" s="7" t="s">
         <v>75</v>
@@ -2129,11 +2131,11 @@
       </c>
       <c r="E37">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F37">
         <f t="shared" si="3"/>
-        <v>2.9726999999999997</v>
+        <v>2.9699999999999998</v>
       </c>
       <c r="K37" s="7" t="s">
         <v>76</v>
@@ -2159,11 +2161,11 @@
       </c>
       <c r="E38">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F38">
         <f t="shared" si="3"/>
-        <v>2.0552000000000001</v>
+        <v>2.0533333333333332</v>
       </c>
       <c r="K38" s="7" t="s">
         <v>77</v>
@@ -2189,11 +2191,11 @@
       </c>
       <c r="E39">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F39">
         <f t="shared" si="3"/>
-        <v>45.764900000000004</v>
+        <v>45.723333333333336</v>
       </c>
       <c r="K39" s="7" t="s">
         <v>78</v>
@@ -2219,11 +2221,11 @@
       </c>
       <c r="E40">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F40">
         <f t="shared" si="3"/>
-        <v>15.414</v>
+        <v>15.4</v>
       </c>
       <c r="K40" s="7" t="s">
         <v>79</v>
@@ -2249,7 +2251,7 @@
       </c>
       <c r="E41">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F41">
         <f t="shared" si="3"/>
@@ -2279,11 +2281,11 @@
       </c>
       <c r="E42">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F42">
         <f t="shared" si="3"/>
-        <v>14.092799999999999</v>
+        <v>14.079999999999998</v>
       </c>
       <c r="K42" s="7" t="s">
         <v>81</v>
@@ -2309,11 +2311,11 @@
       </c>
       <c r="E43">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F43">
         <f t="shared" si="3"/>
-        <v>15.744299999999999</v>
+        <v>15.729999999999999</v>
       </c>
       <c r="K43" s="7" t="s">
         <v>82</v>
@@ -2339,11 +2341,11 @@
       </c>
       <c r="E44">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F44">
         <f t="shared" si="3"/>
-        <v>19.9648</v>
+        <v>19.946666666666669</v>
       </c>
       <c r="K44" s="7" t="s">
         <v>83</v>
@@ -2369,11 +2371,11 @@
       </c>
       <c r="E45">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F45">
         <f t="shared" si="3"/>
-        <v>11.560499999999999</v>
+        <v>11.549999999999999</v>
       </c>
       <c r="K45" s="7" t="s">
         <v>84</v>
@@ -2399,7 +2401,7 @@
       </c>
       <c r="E46">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F46">
         <f t="shared" si="3"/>
@@ -2429,11 +2431,11 @@
       </c>
       <c r="E47">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F47">
         <f t="shared" si="3"/>
-        <v>5.4315999999999995</v>
+        <v>5.4266666666666667</v>
       </c>
       <c r="K47" s="7" t="s">
         <v>86</v>
@@ -2459,11 +2461,11 @@
       </c>
       <c r="E48">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F48">
         <f t="shared" si="3"/>
-        <v>4.1837999999999997</v>
+        <v>4.18</v>
       </c>
       <c r="K48" s="7" t="s">
         <v>87</v>
@@ -2489,11 +2491,11 @@
       </c>
       <c r="E49">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F49">
         <f t="shared" si="3"/>
-        <v>20.038200000000003</v>
+        <v>20.020000000000003</v>
       </c>
       <c r="K49" s="7" t="s">
         <v>88</v>
@@ -2519,11 +2521,11 @@
       </c>
       <c r="E50">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F50">
         <f t="shared" si="3"/>
-        <v>45.508000000000003</v>
+        <v>45.466666666666669</v>
       </c>
       <c r="K50" s="7" t="s">
         <v>89</v>
@@ -2549,11 +2551,11 @@
       </c>
       <c r="E51">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F51">
         <f t="shared" si="3"/>
-        <v>34.6081</v>
+        <v>34.576666666666661</v>
       </c>
       <c r="K51" s="7" t="s">
         <v>90</v>
@@ -2579,11 +2581,11 @@
       </c>
       <c r="E52">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F52">
         <f t="shared" si="3"/>
-        <v>26.203800000000001</v>
+        <v>26.18</v>
       </c>
       <c r="K52" s="7" t="s">
         <v>91</v>
@@ -2609,11 +2611,11 @@
       </c>
       <c r="E53">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F53">
         <f t="shared" si="3"/>
-        <v>26.8277</v>
+        <v>26.803333333333335</v>
       </c>
       <c r="K53" s="7" t="s">
         <v>92</v>
@@ -2639,11 +2641,11 @@
       </c>
       <c r="E54">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F54">
         <f t="shared" si="3"/>
-        <v>12.9184</v>
+        <v>12.906666666666666</v>
       </c>
       <c r="K54" s="7" t="s">
         <v>93</v>
@@ -2669,11 +2671,11 @@
       </c>
       <c r="E55">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F55">
         <f t="shared" si="3"/>
-        <v>18.166499999999999</v>
+        <v>18.149999999999999</v>
       </c>
       <c r="K55" s="7" t="s">
         <v>94</v>
@@ -2699,7 +2701,7 @@
       </c>
       <c r="E56">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F56">
         <f t="shared" si="3"/>
@@ -2729,11 +2731,11 @@
       </c>
       <c r="E57">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F57">
         <f t="shared" si="3"/>
-        <v>3.4498000000000002</v>
+        <v>3.4466666666666668</v>
       </c>
       <c r="K57" s="7" t="s">
         <v>96</v>
@@ -2759,11 +2761,11 @@
       </c>
       <c r="E58">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F58">
         <f t="shared" si="3"/>
-        <v>14.092799999999999</v>
+        <v>14.079999999999998</v>
       </c>
       <c r="K58" s="7" t="s">
         <v>97</v>
@@ -2789,11 +2791,11 @@
       </c>
       <c r="E59">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F59">
         <f t="shared" si="3"/>
-        <v>10.7898</v>
+        <v>10.78</v>
       </c>
       <c r="K59" s="7" t="s">
         <v>98</v>
@@ -2819,11 +2821,11 @@
       </c>
       <c r="E60">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F60">
         <f t="shared" si="3"/>
-        <v>22.02</v>
+        <v>22</v>
       </c>
       <c r="K60" s="7" t="s">
         <v>99</v>
@@ -2849,11 +2851,11 @@
       </c>
       <c r="E61">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F61">
         <f t="shared" si="3"/>
-        <v>13.101900000000001</v>
+        <v>13.09</v>
       </c>
       <c r="K61" s="7" t="s">
         <v>100</v>
@@ -2879,11 +2881,11 @@
       </c>
       <c r="E62">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F62">
         <f t="shared" si="3"/>
-        <v>24.809199999999997</v>
+        <v>24.786666666666665</v>
       </c>
       <c r="K62" s="7" t="s">
         <v>101</v>
@@ -2909,7 +2911,7 @@
       </c>
       <c r="E63">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F63">
         <f t="shared" si="3"/>
@@ -2939,11 +2941,11 @@
       </c>
       <c r="E64">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F64">
         <f t="shared" si="3"/>
-        <v>47.563199999999995</v>
+        <v>47.519999999999996</v>
       </c>
       <c r="K64" s="7" t="s">
         <v>103</v>
@@ -2969,11 +2971,11 @@
       </c>
       <c r="E65">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F65">
         <f t="shared" si="3"/>
-        <v>64.591999999999999</v>
+        <v>64.533333333333331</v>
       </c>
       <c r="K65" s="7" t="s">
         <v>104</v>
@@ -2999,7 +3001,7 @@
       </c>
       <c r="E66">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F66">
         <f t="shared" si="3"/>
@@ -3029,7 +3031,7 @@
       </c>
       <c r="E67">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F67">
         <f t="shared" si="3"/>
@@ -3059,11 +3061,11 @@
       </c>
       <c r="E68">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F68">
         <f t="shared" si="3"/>
-        <v>21.286000000000001</v>
+        <v>21.266666666666669</v>
       </c>
       <c r="K68" s="7" t="s">
         <v>107</v>
@@ -3089,11 +3091,11 @@
       </c>
       <c r="E69">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F69">
         <f t="shared" si="3"/>
-        <v>71.454900000000009</v>
+        <v>71.39</v>
       </c>
       <c r="K69" s="7" t="s">
         <v>108</v>
@@ -3119,7 +3121,7 @@
       </c>
       <c r="E70">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F70">
         <f t="shared" si="3"/>
@@ -3149,11 +3151,11 @@
       </c>
       <c r="E71">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F71">
         <f t="shared" si="3"/>
-        <v>11.1935</v>
+        <v>11.183333333333334</v>
       </c>
       <c r="K71" s="7" t="s">
         <v>110</v>
@@ -3179,11 +3181,11 @@
       </c>
       <c r="E72">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F72">
         <f t="shared" si="3"/>
-        <v>59.160400000000003</v>
+        <v>59.106666666666669</v>
       </c>
       <c r="K72" s="7" t="s">
         <v>111</v>
@@ -3209,11 +3211,11 @@
       </c>
       <c r="E73">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F73">
         <f t="shared" si="3"/>
-        <v>60.114599999999996</v>
+        <v>60.059999999999995</v>
       </c>
       <c r="K73" s="7" t="s">
         <v>112</v>
@@ -3239,11 +3241,11 @@
       </c>
       <c r="E74">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F74">
         <f t="shared" si="3"/>
-        <v>7.0463999999999993</v>
+        <v>7.0399999999999991</v>
       </c>
       <c r="K74" s="7" t="s">
         <v>113</v>
@@ -3269,11 +3271,11 @@
       </c>
       <c r="E75">
         <f t="shared" si="2"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F75">
         <f t="shared" si="3"/>
-        <v>88.263500000000008</v>
+        <v>88.183333333333337</v>
       </c>
       <c r="K75" s="7" t="s">
         <v>114</v>
@@ -3299,11 +3301,11 @@
       </c>
       <c r="E76">
         <f t="shared" ref="E76:E94" si="6">$M$7</f>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F76">
         <f t="shared" ref="F76:F94" si="7">D76*E76*-1</f>
-        <v>2.4222000000000001</v>
+        <v>2.42</v>
       </c>
       <c r="K76" s="7" t="s">
         <v>115</v>
@@ -3329,11 +3331,11 @@
       </c>
       <c r="E77">
         <f t="shared" si="6"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F77">
         <f t="shared" si="7"/>
-        <v>7.3766999999999987</v>
+        <v>7.3699999999999992</v>
       </c>
       <c r="K77" s="7" t="s">
         <v>116</v>
@@ -3359,11 +3361,11 @@
       </c>
       <c r="E78">
         <f t="shared" si="6"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F78">
         <f t="shared" si="7"/>
-        <v>24.956000000000003</v>
+        <v>24.933333333333334</v>
       </c>
       <c r="K78" s="7" t="s">
         <v>117</v>
@@ -3389,11 +3391,11 @@
       </c>
       <c r="E79">
         <f t="shared" si="6"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F79">
         <f t="shared" si="7"/>
-        <v>63.307499999999997</v>
+        <v>63.25</v>
       </c>
       <c r="K79" s="7" t="s">
         <v>118</v>
@@ -3419,11 +3421,11 @@
       </c>
       <c r="E80">
         <f t="shared" si="6"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F80">
         <f t="shared" si="7"/>
-        <v>69.363</v>
+        <v>69.300000000000011</v>
       </c>
       <c r="K80" s="7" t="s">
         <v>119</v>
@@ -3449,11 +3451,11 @@
       </c>
       <c r="E81">
         <f t="shared" si="6"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F81">
         <f t="shared" si="7"/>
-        <v>46.9026</v>
+        <v>46.859999999999992</v>
       </c>
       <c r="K81" s="7" t="s">
         <v>120</v>
@@ -3479,11 +3481,11 @@
       </c>
       <c r="E82">
         <f t="shared" si="6"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F82">
         <f t="shared" si="7"/>
-        <v>31.7088</v>
+        <v>31.68</v>
       </c>
       <c r="K82" s="7" t="s">
         <v>121</v>
@@ -3509,11 +3511,11 @@
       </c>
       <c r="E83">
         <f t="shared" si="6"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F83">
         <f t="shared" si="7"/>
-        <v>58.940199999999997</v>
+        <v>58.886666666666656</v>
       </c>
       <c r="K83" s="7" t="s">
         <v>122</v>
@@ -3539,11 +3541,11 @@
       </c>
       <c r="E84">
         <f t="shared" si="6"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F84">
         <f t="shared" si="7"/>
-        <v>54.316000000000003</v>
+        <v>54.266666666666666</v>
       </c>
       <c r="K84" s="7" t="s">
         <v>123</v>
@@ -3569,11 +3571,11 @@
       </c>
       <c r="E85">
         <f t="shared" si="6"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F85">
         <f t="shared" si="7"/>
-        <v>49.545000000000002</v>
+        <v>49.5</v>
       </c>
       <c r="K85" s="7" t="s">
         <v>124</v>
@@ -3599,11 +3601,11 @@
       </c>
       <c r="E86">
         <f t="shared" si="6"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F86">
         <f t="shared" si="7"/>
-        <v>111.56800000000001</v>
+        <v>111.46666666666667</v>
       </c>
       <c r="K86" s="7" t="s">
         <v>125</v>
@@ -3629,11 +3631,11 @@
       </c>
       <c r="E87">
         <f t="shared" si="6"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F87">
         <f t="shared" si="7"/>
-        <v>59.343899999999991</v>
+        <v>59.289999999999992</v>
       </c>
       <c r="K87" s="7" t="s">
         <v>126</v>
@@ -3659,11 +3661,11 @@
       </c>
       <c r="E88">
         <f t="shared" si="6"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F88">
         <f t="shared" si="7"/>
-        <v>111.6414</v>
+        <v>111.54</v>
       </c>
       <c r="K88" s="7" t="s">
         <v>127</v>
@@ -3689,11 +3691,11 @@
       </c>
       <c r="E89">
         <f t="shared" si="6"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F89">
         <f t="shared" si="7"/>
-        <v>200.05169999999998</v>
+        <v>199.86999999999998</v>
       </c>
       <c r="K89" s="7" t="s">
         <v>128</v>
@@ -3719,7 +3721,7 @@
       </c>
       <c r="E90">
         <f t="shared" si="6"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F90">
         <f t="shared" si="7"/>
@@ -3749,11 +3751,11 @@
       </c>
       <c r="E91">
         <f t="shared" si="6"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F91">
         <f t="shared" si="7"/>
-        <v>20.808900000000001</v>
+        <v>20.790000000000003</v>
       </c>
       <c r="K91" s="7" t="s">
         <v>130</v>
@@ -3779,11 +3781,11 @@
       </c>
       <c r="E92">
         <f t="shared" si="6"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F92">
         <f t="shared" si="7"/>
-        <v>171.53579999999997</v>
+        <v>171.37999999999997</v>
       </c>
       <c r="K92" s="7" t="s">
         <v>131</v>
@@ -3809,11 +3811,11 @@
       </c>
       <c r="E93">
         <f t="shared" si="6"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F93">
         <f t="shared" si="7"/>
-        <v>204.08870000000002</v>
+        <v>203.90333333333334</v>
       </c>
       <c r="K93" s="7" t="s">
         <v>132</v>
@@ -3839,11 +3841,11 @@
       </c>
       <c r="E94">
         <f t="shared" si="6"/>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="F94">
         <f t="shared" si="7"/>
-        <v>15.414</v>
+        <v>15.4</v>
       </c>
       <c r="K94" s="7" t="s">
         <v>133</v>
@@ -3880,7 +3882,8 @@
         <v>23</v>
       </c>
       <c r="G7">
-        <v>3.67</v>
+        <f>44/12</f>
+        <v>3.6666666666666665</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -3917,11 +3920,11 @@
       </c>
       <c r="C11">
         <f>$G$7</f>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="D11">
         <f>A11*B11*C11*-1</f>
-        <v>-642.25</v>
+        <v>-641.66666666666663</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -3933,11 +3936,11 @@
       </c>
       <c r="C12">
         <f>$G$7</f>
-        <v>3.67</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="D12">
         <f>A12*B12*C12*-1</f>
-        <v>-292.42560000000003</v>
+        <v>-292.16000000000003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(calculators): lulucf updates after working on fullcam layer
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/16-lulucf/16.1-lulucf.xlsx
+++ b/packages/calculators/src/modules/test/16-lulucf/16.1-lulucf.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/16-lulucf/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{467B2523-29EF-0742-9B74-29AC65CA6F22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB847984-2549-C142-8149-702321047583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51200" yWindow="13240" windowWidth="28800" windowHeight="27420" activeTab="3" xr2:uid="{CC0FEAF9-C40F-694B-BCB9-117AFB86C05D}"/>
+    <workbookView xWindow="51200" yWindow="13240" windowWidth="28800" windowHeight="27420" activeTab="1" xr2:uid="{CC0FEAF9-C40F-694B-BCB9-117AFB86C05D}"/>
   </bookViews>
   <sheets>
     <sheet name="16.1.1.2" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="139">
   <si>
     <t>Scenario</t>
   </si>
@@ -152,22 +152,13 @@
     <t>Deforesting</t>
   </si>
   <si>
-    <t>Egijy</t>
-  </si>
-  <si>
     <t>agijy</t>
   </si>
   <si>
-    <t>ELUCgjy</t>
-  </si>
-  <si>
     <t>Emissions from biomass burning</t>
   </si>
   <si>
     <t>t CO2e</t>
-  </si>
-  <si>
-    <t>t CO2e / ha</t>
   </si>
   <si>
     <t>Area burnt</t>
@@ -518,6 +509,30 @@
   </si>
   <si>
     <t>Yalgoo</t>
+  </si>
+  <si>
+    <t>Eg=ch4,I,j,y</t>
+  </si>
+  <si>
+    <t>t CH4 / ha</t>
+  </si>
+  <si>
+    <t>t N2O / ha</t>
+  </si>
+  <si>
+    <t>Eg=n2o,I,j,y</t>
+  </si>
+  <si>
+    <t>ELUCg=ch4jy</t>
+  </si>
+  <si>
+    <t>t CH4</t>
+  </si>
+  <si>
+    <t>t N2O</t>
+  </si>
+  <si>
+    <t>ELUCg=n2ojy</t>
   </si>
 </sst>
 </file>
@@ -946,16 +961,16 @@
   <sheetData>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -1161,64 +1176,89 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92CDB52C-734F-7046-ACDC-C5573D991542}">
-  <dimension ref="A4:D13"/>
+  <dimension ref="A4:F13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="16.1640625" customWidth="1"/>
-    <col min="3" max="3" width="18.1640625" customWidth="1"/>
-    <col min="4" max="4" width="19.33203125" customWidth="1"/>
+    <col min="2" max="3" width="16.1640625" customWidth="1"/>
+    <col min="4" max="4" width="18.1640625" customWidth="1"/>
+    <col min="5" max="5" width="19.33203125" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+      <c r="C4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>5</v>
       </c>
       <c r="C6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>31</v>
+        <v>132</v>
       </c>
       <c r="C7" t="s">
+        <v>133</v>
+      </c>
+      <c r="D7" t="s">
         <v>24</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
+        <v>136</v>
+      </c>
+      <c r="F7" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="B9" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B9" s="1" t="s">
-        <v>33</v>
-      </c>
       <c r="C9" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>0</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E10" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -1226,16 +1266,23 @@
         <v>25</v>
       </c>
       <c r="C11">
+        <v>4</v>
+      </c>
+      <c r="D11">
         <v>5</v>
       </c>
-      <c r="D11">
-        <f>B11*C11</f>
+      <c r="E11">
+        <f>B11*D11</f>
         <v>125</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="F11">
+        <f>C11*D11</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -1244,23 +1291,37 @@
         <v>0</v>
       </c>
       <c r="D12">
-        <f t="shared" ref="D12:D13" si="0">B12*C12</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <f t="shared" ref="E12:F13" si="0">B12*D12</f>
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <f t="shared" ref="F12:F13" si="1">C12*D12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B13">
         <v>35</v>
       </c>
       <c r="C13">
+        <v>40</v>
+      </c>
+      <c r="D13">
         <v>200</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <f t="shared" si="0"/>
         <v>7000</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="1"/>
+        <v>8000</v>
       </c>
     </row>
   </sheetData>
@@ -1287,10 +1348,10 @@
         <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="L7" t="s">
         <v>23</v>
@@ -1305,38 +1366,38 @@
         <v>19</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E10" t="s">
         <v>23</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -1358,7 +1419,7 @@
         <v>0.43999999999999995</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="L11" s="7">
         <v>-0.12</v>
@@ -1366,7 +1427,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B12">
         <v>2</v>
@@ -1388,7 +1449,7 @@
         <v>2.86</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="L12" s="7">
         <v>-0.39</v>
@@ -1396,7 +1457,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B13">
         <v>3</v>
@@ -1418,7 +1479,7 @@
         <v>0.99</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="L13" s="7">
         <v>-0.09</v>
@@ -1426,7 +1487,7 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B14">
         <v>4</v>
@@ -1448,7 +1509,7 @@
         <v>1.3199999999999998</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="L14" s="7">
         <v>-0.09</v>
@@ -1456,7 +1517,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B15">
         <v>5</v>
@@ -1478,7 +1539,7 @@
         <v>2.3833333333333333</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="L15" s="7">
         <v>-0.13</v>
@@ -1486,7 +1547,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B16">
         <v>6</v>
@@ -1508,7 +1569,7 @@
         <v>2.86</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L16" s="7">
         <v>-0.13</v>
@@ -1516,7 +1577,7 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B17">
         <v>7</v>
@@ -1538,7 +1599,7 @@
         <v>14.116666666666669</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="L17" s="7">
         <v>-0.55000000000000004</v>
@@ -1546,7 +1607,7 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B18">
         <v>8</v>
@@ -1568,7 +1629,7 @@
         <v>0.29333333333333333</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="L18" s="7">
         <v>-0.01</v>
@@ -1576,7 +1637,7 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B19">
         <v>9</v>
@@ -1598,7 +1659,7 @@
         <v>2.3100000000000005</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="L19" s="7">
         <v>-7.0000000000000007E-2</v>
@@ -1606,7 +1667,7 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B20">
         <v>10</v>
@@ -1628,7 +1689,7 @@
         <v>2.1999999999999997</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="L20" s="7">
         <v>-0.06</v>
@@ -1636,7 +1697,7 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B21">
         <v>11</v>
@@ -1658,7 +1719,7 @@
         <v>3.63</v>
       </c>
       <c r="K21" s="7" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="L21" s="7">
         <v>-0.09</v>
@@ -1666,7 +1727,7 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B22">
         <v>12</v>
@@ -1688,7 +1749,7 @@
         <v>8.3600000000000012</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="L22" s="7">
         <v>-0.19</v>
@@ -1696,7 +1757,7 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B23">
         <v>13</v>
@@ -1718,7 +1779,7 @@
         <v>6.1966666666666663</v>
       </c>
       <c r="K23" s="7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L23" s="7">
         <v>-0.13</v>
@@ -1726,7 +1787,7 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B24">
         <v>14</v>
@@ -1748,7 +1809,7 @@
         <v>2.0533333333333332</v>
       </c>
       <c r="K24" s="7" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L24" s="7">
         <v>-0.04</v>
@@ -1756,7 +1817,7 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B25">
         <v>15</v>
@@ -1778,7 +1839,7 @@
         <v>22</v>
       </c>
       <c r="K25" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="L25" s="7">
         <v>-0.4</v>
@@ -1786,7 +1847,7 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B26">
         <v>16</v>
@@ -1808,7 +1869,7 @@
         <v>5.2799999999999994</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="L26" s="7">
         <v>-0.09</v>
@@ -1816,7 +1877,7 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B27">
         <v>17</v>
@@ -1838,7 +1899,7 @@
         <v>0</v>
       </c>
       <c r="K27" s="7" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="L27" s="7">
         <v>0</v>
@@ -1846,7 +1907,7 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B28">
         <v>18</v>
@@ -1868,7 +1929,7 @@
         <v>29.04</v>
       </c>
       <c r="K28" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="L28" s="7">
         <v>-0.44</v>
@@ -1876,7 +1937,7 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B29">
         <v>19</v>
@@ -1898,7 +1959,7 @@
         <v>14.629999999999999</v>
       </c>
       <c r="K29" s="7" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="L29" s="7">
         <v>-0.21</v>
@@ -1906,7 +1967,7 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B30">
         <v>20</v>
@@ -1928,7 +1989,7 @@
         <v>15.4</v>
       </c>
       <c r="K30" s="7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="L30" s="7">
         <v>-0.21</v>
@@ -1936,7 +1997,7 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B31">
         <v>21</v>
@@ -1958,7 +2019,7 @@
         <v>0</v>
       </c>
       <c r="K31" s="7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="L31" s="7">
         <v>0</v>
@@ -1966,7 +2027,7 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B32">
         <v>22</v>
@@ -1988,7 +2049,7 @@
         <v>3.2266666666666666</v>
       </c>
       <c r="K32" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="L32" s="7">
         <v>-0.04</v>
@@ -1996,7 +2057,7 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B33">
         <v>23</v>
@@ -2018,7 +2079,7 @@
         <v>5.9033333333333333</v>
       </c>
       <c r="K33" s="7" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="L33" s="7">
         <v>-7.0000000000000007E-2</v>
@@ -2026,7 +2087,7 @@
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" s="7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B34">
         <v>24</v>
@@ -2048,7 +2109,7 @@
         <v>3.5199999999999996</v>
       </c>
       <c r="K34" s="7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="L34" s="7">
         <v>-0.04</v>
@@ -2056,7 +2117,7 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" s="7" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B35">
         <v>25</v>
@@ -2078,7 +2139,7 @@
         <v>22</v>
       </c>
       <c r="K35" s="7" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="L35" s="7">
         <v>-0.24</v>
@@ -2086,7 +2147,7 @@
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" s="7" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B36">
         <v>26</v>
@@ -2108,7 +2169,7 @@
         <v>16.206666666666667</v>
       </c>
       <c r="K36" s="7" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="L36" s="7">
         <v>-0.17</v>
@@ -2116,7 +2177,7 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B37">
         <v>27</v>
@@ -2138,7 +2199,7 @@
         <v>2.9699999999999998</v>
       </c>
       <c r="K37" s="7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="L37" s="7">
         <v>-0.03</v>
@@ -2146,7 +2207,7 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B38">
         <v>28</v>
@@ -2168,7 +2229,7 @@
         <v>2.0533333333333332</v>
       </c>
       <c r="K38" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="L38" s="7">
         <v>-0.02</v>
@@ -2176,7 +2237,7 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" s="7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B39">
         <v>29</v>
@@ -2198,7 +2259,7 @@
         <v>45.723333333333336</v>
       </c>
       <c r="K39" s="7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="L39" s="7">
         <v>-0.43</v>
@@ -2206,7 +2267,7 @@
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B40">
         <v>30</v>
@@ -2228,7 +2289,7 @@
         <v>15.4</v>
       </c>
       <c r="K40" s="7" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="L40" s="7">
         <v>-0.14000000000000001</v>
@@ -2236,7 +2297,7 @@
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" s="7" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B41">
         <v>31</v>
@@ -2258,7 +2319,7 @@
         <v>0</v>
       </c>
       <c r="K41" s="7" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="L41" s="7">
         <v>0</v>
@@ -2266,7 +2327,7 @@
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B42">
         <v>32</v>
@@ -2288,7 +2349,7 @@
         <v>14.079999999999998</v>
       </c>
       <c r="K42" s="7" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="L42" s="7">
         <v>-0.12</v>
@@ -2296,7 +2357,7 @@
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" s="7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B43">
         <v>33</v>
@@ -2318,7 +2379,7 @@
         <v>15.729999999999999</v>
       </c>
       <c r="K43" s="7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="L43" s="7">
         <v>-0.13</v>
@@ -2326,7 +2387,7 @@
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44" s="7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B44">
         <v>34</v>
@@ -2348,7 +2409,7 @@
         <v>19.946666666666669</v>
       </c>
       <c r="K44" s="7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="L44" s="7">
         <v>-0.16</v>
@@ -2356,7 +2417,7 @@
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A45" s="7" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B45">
         <v>35</v>
@@ -2378,7 +2439,7 @@
         <v>11.549999999999999</v>
       </c>
       <c r="K45" s="7" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="L45" s="7">
         <v>-0.09</v>
@@ -2386,7 +2447,7 @@
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46" s="7" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B46">
         <v>36</v>
@@ -2408,7 +2469,7 @@
         <v>0</v>
       </c>
       <c r="K46" s="7" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="L46" s="7">
         <v>0</v>
@@ -2416,7 +2477,7 @@
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A47" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B47">
         <v>37</v>
@@ -2438,7 +2499,7 @@
         <v>5.4266666666666667</v>
       </c>
       <c r="K47" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="L47" s="7">
         <v>-0.04</v>
@@ -2446,7 +2507,7 @@
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48" s="7" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B48">
         <v>38</v>
@@ -2468,7 +2529,7 @@
         <v>4.18</v>
       </c>
       <c r="K48" s="7" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="L48" s="7">
         <v>-0.03</v>
@@ -2476,7 +2537,7 @@
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B49">
         <v>39</v>
@@ -2498,7 +2559,7 @@
         <v>20.020000000000003</v>
       </c>
       <c r="K49" s="7" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="L49" s="7">
         <v>-0.14000000000000001</v>
@@ -2506,7 +2567,7 @@
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A50" s="7" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B50">
         <v>40</v>
@@ -2528,7 +2589,7 @@
         <v>45.466666666666669</v>
       </c>
       <c r="K50" s="7" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L50" s="7">
         <v>-0.31</v>
@@ -2536,7 +2597,7 @@
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B51">
         <v>41</v>
@@ -2558,7 +2619,7 @@
         <v>34.576666666666661</v>
       </c>
       <c r="K51" s="7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="L51" s="7">
         <v>-0.23</v>
@@ -2566,7 +2627,7 @@
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A52" s="7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B52">
         <v>42</v>
@@ -2588,7 +2649,7 @@
         <v>26.18</v>
       </c>
       <c r="K52" s="7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L52" s="7">
         <v>-0.17</v>
@@ -2596,7 +2657,7 @@
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B53">
         <v>43</v>
@@ -2618,7 +2679,7 @@
         <v>26.803333333333335</v>
       </c>
       <c r="K53" s="7" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="L53" s="7">
         <v>-0.17</v>
@@ -2626,7 +2687,7 @@
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A54" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B54">
         <v>44</v>
@@ -2648,7 +2709,7 @@
         <v>12.906666666666666</v>
       </c>
       <c r="K54" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="L54" s="7">
         <v>-0.08</v>
@@ -2656,7 +2717,7 @@
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B55">
         <v>45</v>
@@ -2678,7 +2739,7 @@
         <v>18.149999999999999</v>
       </c>
       <c r="K55" s="7" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="L55" s="7">
         <v>-0.11</v>
@@ -2686,7 +2747,7 @@
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A56" s="7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B56">
         <v>46</v>
@@ -2708,7 +2769,7 @@
         <v>0</v>
       </c>
       <c r="K56" s="7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="L56" s="7">
         <v>0</v>
@@ -2716,7 +2777,7 @@
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A57" s="7" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B57">
         <v>47</v>
@@ -2738,7 +2799,7 @@
         <v>3.4466666666666668</v>
       </c>
       <c r="K57" s="7" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="L57" s="7">
         <v>-0.02</v>
@@ -2746,7 +2807,7 @@
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B58">
         <v>48</v>
@@ -2768,7 +2829,7 @@
         <v>14.079999999999998</v>
       </c>
       <c r="K58" s="7" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="L58" s="7">
         <v>-0.08</v>
@@ -2776,7 +2837,7 @@
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A59" s="7" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B59">
         <v>49</v>
@@ -2798,7 +2859,7 @@
         <v>10.78</v>
       </c>
       <c r="K59" s="7" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="L59" s="7">
         <v>-0.06</v>
@@ -2806,7 +2867,7 @@
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A60" s="7" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B60">
         <v>50</v>
@@ -2828,7 +2889,7 @@
         <v>22</v>
       </c>
       <c r="K60" s="7" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="L60" s="7">
         <v>-0.12</v>
@@ -2836,7 +2897,7 @@
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A61" s="7" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B61">
         <v>51</v>
@@ -2858,7 +2919,7 @@
         <v>13.09</v>
       </c>
       <c r="K61" s="7" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="L61" s="7">
         <v>-7.0000000000000007E-2</v>
@@ -2866,7 +2927,7 @@
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62" s="7" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B62">
         <v>52</v>
@@ -2888,7 +2949,7 @@
         <v>24.786666666666665</v>
       </c>
       <c r="K62" s="7" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="L62" s="7">
         <v>-0.13</v>
@@ -2896,7 +2957,7 @@
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B63">
         <v>53</v>
@@ -2918,7 +2979,7 @@
         <v>0</v>
       </c>
       <c r="K63" s="7" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="L63" s="7">
         <v>0</v>
@@ -2926,7 +2987,7 @@
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" s="7" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B64">
         <v>54</v>
@@ -2948,7 +3009,7 @@
         <v>47.519999999999996</v>
       </c>
       <c r="K64" s="7" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="L64" s="7">
         <v>-0.24</v>
@@ -2956,7 +3017,7 @@
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A65" s="7" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B65">
         <v>55</v>
@@ -2978,7 +3039,7 @@
         <v>64.533333333333331</v>
       </c>
       <c r="K65" s="7" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="L65" s="7">
         <v>-0.32</v>
@@ -2986,7 +3047,7 @@
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A66" s="7" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B66">
         <v>56</v>
@@ -3008,7 +3069,7 @@
         <v>0</v>
       </c>
       <c r="K66" s="7" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="L66" s="7">
         <v>0</v>
@@ -3016,7 +3077,7 @@
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B67">
         <v>57</v>
@@ -3038,7 +3099,7 @@
         <v>0</v>
       </c>
       <c r="K67" s="7" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="L67" s="7">
         <v>0</v>
@@ -3046,7 +3107,7 @@
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A68" s="7" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B68">
         <v>58</v>
@@ -3068,7 +3129,7 @@
         <v>21.266666666666669</v>
       </c>
       <c r="K68" s="7" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="L68" s="7">
         <v>-0.1</v>
@@ -3076,7 +3137,7 @@
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A69" s="7" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B69">
         <v>59</v>
@@ -3098,7 +3159,7 @@
         <v>71.39</v>
       </c>
       <c r="K69" s="7" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="L69" s="7">
         <v>-0.33</v>
@@ -3106,7 +3167,7 @@
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A70" s="7" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B70">
         <v>60</v>
@@ -3128,7 +3189,7 @@
         <v>0</v>
       </c>
       <c r="K70" s="7" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="L70" s="7">
         <v>0</v>
@@ -3136,7 +3197,7 @@
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A71" s="7" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B71">
         <v>61</v>
@@ -3158,7 +3219,7 @@
         <v>11.183333333333334</v>
       </c>
       <c r="K71" s="7" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="L71" s="7">
         <v>-0.05</v>
@@ -3166,7 +3227,7 @@
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A72" s="7" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B72">
         <v>62</v>
@@ -3188,7 +3249,7 @@
         <v>59.106666666666669</v>
       </c>
       <c r="K72" s="7" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="L72" s="7">
         <v>-0.26</v>
@@ -3196,7 +3257,7 @@
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A73" s="7" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B73">
         <v>63</v>
@@ -3218,7 +3279,7 @@
         <v>60.059999999999995</v>
       </c>
       <c r="K73" s="7" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="L73" s="7">
         <v>-0.26</v>
@@ -3226,7 +3287,7 @@
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A74" s="7" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B74">
         <v>64</v>
@@ -3248,7 +3309,7 @@
         <v>7.0399999999999991</v>
       </c>
       <c r="K74" s="7" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="L74" s="7">
         <v>-0.03</v>
@@ -3256,7 +3317,7 @@
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A75" s="7" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B75">
         <v>65</v>
@@ -3278,7 +3339,7 @@
         <v>88.183333333333337</v>
       </c>
       <c r="K75" s="7" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="L75" s="7">
         <v>-0.37</v>
@@ -3286,7 +3347,7 @@
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B76">
         <v>66</v>
@@ -3308,7 +3369,7 @@
         <v>2.42</v>
       </c>
       <c r="K76" s="7" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="L76" s="7">
         <v>-0.01</v>
@@ -3316,7 +3377,7 @@
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A77" s="7" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B77">
         <v>67</v>
@@ -3338,7 +3399,7 @@
         <v>7.3699999999999992</v>
       </c>
       <c r="K77" s="7" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="L77" s="7">
         <v>-0.03</v>
@@ -3346,7 +3407,7 @@
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A78" s="7" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B78">
         <v>68</v>
@@ -3368,7 +3429,7 @@
         <v>24.933333333333334</v>
       </c>
       <c r="K78" s="7" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="L78" s="7">
         <v>-0.1</v>
@@ -3376,7 +3437,7 @@
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A79" s="7" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B79">
         <v>69</v>
@@ -3398,7 +3459,7 @@
         <v>63.25</v>
       </c>
       <c r="K79" s="7" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="L79" s="7">
         <v>-0.25</v>
@@ -3406,7 +3467,7 @@
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A80" s="7" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B80">
         <v>70</v>
@@ -3428,7 +3489,7 @@
         <v>69.300000000000011</v>
       </c>
       <c r="K80" s="7" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="L80" s="7">
         <v>-0.27</v>
@@ -3436,7 +3497,7 @@
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A81" s="7" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B81">
         <v>71</v>
@@ -3458,7 +3519,7 @@
         <v>46.859999999999992</v>
       </c>
       <c r="K81" s="7" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="L81" s="7">
         <v>-0.18</v>
@@ -3466,7 +3527,7 @@
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A82" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B82">
         <v>72</v>
@@ -3488,7 +3549,7 @@
         <v>31.68</v>
       </c>
       <c r="K82" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="L82" s="7">
         <v>-0.12</v>
@@ -3496,7 +3557,7 @@
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A83" s="7" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B83">
         <v>73</v>
@@ -3518,7 +3579,7 @@
         <v>58.886666666666656</v>
       </c>
       <c r="K83" s="7" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="L83" s="7">
         <v>-0.22</v>
@@ -3526,7 +3587,7 @@
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A84" s="7" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B84">
         <v>74</v>
@@ -3548,7 +3609,7 @@
         <v>54.266666666666666</v>
       </c>
       <c r="K84" s="7" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="L84" s="7">
         <v>-0.2</v>
@@ -3556,7 +3617,7 @@
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B85">
         <v>75</v>
@@ -3578,7 +3639,7 @@
         <v>49.5</v>
       </c>
       <c r="K85" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="L85" s="7">
         <v>-0.18</v>
@@ -3586,7 +3647,7 @@
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A86" s="7" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B86">
         <v>76</v>
@@ -3608,7 +3669,7 @@
         <v>111.46666666666667</v>
       </c>
       <c r="K86" s="7" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="L86" s="7">
         <v>-0.4</v>
@@ -3616,7 +3677,7 @@
     </row>
     <row r="87" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A87" s="7" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B87">
         <v>77</v>
@@ -3638,7 +3699,7 @@
         <v>59.289999999999992</v>
       </c>
       <c r="K87" s="7" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="L87" s="7">
         <v>-0.21</v>
@@ -3646,7 +3707,7 @@
     </row>
     <row r="88" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A88" s="7" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B88">
         <v>78</v>
@@ -3668,7 +3729,7 @@
         <v>111.54</v>
       </c>
       <c r="K88" s="7" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="L88" s="7">
         <v>-0.39</v>
@@ -3676,7 +3737,7 @@
     </row>
     <row r="89" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A89" s="7" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B89">
         <v>79</v>
@@ -3698,7 +3759,7 @@
         <v>199.86999999999998</v>
       </c>
       <c r="K89" s="7" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="L89" s="7">
         <v>-0.69</v>
@@ -3706,7 +3767,7 @@
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A90" s="7" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B90">
         <v>80</v>
@@ -3728,7 +3789,7 @@
         <v>0</v>
       </c>
       <c r="K90" s="7" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="L90" s="7">
         <v>0</v>
@@ -3736,7 +3797,7 @@
     </row>
     <row r="91" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A91" s="7" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B91">
         <v>81</v>
@@ -3758,7 +3819,7 @@
         <v>20.790000000000003</v>
       </c>
       <c r="K91" s="7" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="L91" s="7">
         <v>-7.0000000000000007E-2</v>
@@ -3766,7 +3827,7 @@
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A92" s="7" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B92">
         <v>82</v>
@@ -3788,7 +3849,7 @@
         <v>171.37999999999997</v>
       </c>
       <c r="K92" s="7" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="L92" s="7">
         <v>-0.56999999999999995</v>
@@ -3796,7 +3857,7 @@
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A93" s="7" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B93">
         <v>83</v>
@@ -3818,7 +3879,7 @@
         <v>203.90333333333334</v>
       </c>
       <c r="K93" s="7" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="L93" s="7">
         <v>-0.67</v>
@@ -3826,7 +3887,7 @@
     </row>
     <row r="94" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A94" s="7" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B94">
         <v>84</v>
@@ -3848,7 +3909,7 @@
         <v>15.4</v>
       </c>
       <c r="K94" s="7" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="L94" s="7">
         <v>-0.05</v>
@@ -3866,7 +3927,7 @@
   <sheetData>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -3894,21 +3955,21 @@
         <v>24</v>
       </c>
       <c r="D8" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C10" t="s">
         <v>23</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Changes to the public package API to prepare for exposing v4 of the API (#193)
* feat(calculators): changes to allow making FullCAM API requests outside of the NPM package
* feat(calculators): changes needed to get beta package running in API
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/16-lulucf/16.1-lulucf.xlsx
+++ b/packages/calculators/src/modules/test/16-lulucf/16.1-lulucf.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/16-lulucf/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{467B2523-29EF-0742-9B74-29AC65CA6F22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB847984-2549-C142-8149-702321047583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51200" yWindow="13240" windowWidth="28800" windowHeight="27420" activeTab="3" xr2:uid="{CC0FEAF9-C40F-694B-BCB9-117AFB86C05D}"/>
+    <workbookView xWindow="51200" yWindow="13240" windowWidth="28800" windowHeight="27420" activeTab="1" xr2:uid="{CC0FEAF9-C40F-694B-BCB9-117AFB86C05D}"/>
   </bookViews>
   <sheets>
     <sheet name="16.1.1.2" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="139">
   <si>
     <t>Scenario</t>
   </si>
@@ -152,22 +152,13 @@
     <t>Deforesting</t>
   </si>
   <si>
-    <t>Egijy</t>
-  </si>
-  <si>
     <t>agijy</t>
   </si>
   <si>
-    <t>ELUCgjy</t>
-  </si>
-  <si>
     <t>Emissions from biomass burning</t>
   </si>
   <si>
     <t>t CO2e</t>
-  </si>
-  <si>
-    <t>t CO2e / ha</t>
   </si>
   <si>
     <t>Area burnt</t>
@@ -518,6 +509,30 @@
   </si>
   <si>
     <t>Yalgoo</t>
+  </si>
+  <si>
+    <t>Eg=ch4,I,j,y</t>
+  </si>
+  <si>
+    <t>t CH4 / ha</t>
+  </si>
+  <si>
+    <t>t N2O / ha</t>
+  </si>
+  <si>
+    <t>Eg=n2o,I,j,y</t>
+  </si>
+  <si>
+    <t>ELUCg=ch4jy</t>
+  </si>
+  <si>
+    <t>t CH4</t>
+  </si>
+  <si>
+    <t>t N2O</t>
+  </si>
+  <si>
+    <t>ELUCg=n2ojy</t>
   </si>
 </sst>
 </file>
@@ -946,16 +961,16 @@
   <sheetData>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -1161,64 +1176,89 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92CDB52C-734F-7046-ACDC-C5573D991542}">
-  <dimension ref="A4:D13"/>
+  <dimension ref="A4:F13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="16.1640625" customWidth="1"/>
-    <col min="3" max="3" width="18.1640625" customWidth="1"/>
-    <col min="4" max="4" width="19.33203125" customWidth="1"/>
+    <col min="2" max="3" width="16.1640625" customWidth="1"/>
+    <col min="4" max="4" width="18.1640625" customWidth="1"/>
+    <col min="5" max="5" width="19.33203125" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+      <c r="C4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>5</v>
       </c>
       <c r="C6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>31</v>
+        <v>132</v>
       </c>
       <c r="C7" t="s">
+        <v>133</v>
+      </c>
+      <c r="D7" t="s">
         <v>24</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
+        <v>136</v>
+      </c>
+      <c r="F7" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="B9" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B9" s="1" t="s">
-        <v>33</v>
-      </c>
       <c r="C9" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>0</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E10" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -1226,16 +1266,23 @@
         <v>25</v>
       </c>
       <c r="C11">
+        <v>4</v>
+      </c>
+      <c r="D11">
         <v>5</v>
       </c>
-      <c r="D11">
-        <f>B11*C11</f>
+      <c r="E11">
+        <f>B11*D11</f>
         <v>125</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="F11">
+        <f>C11*D11</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -1244,23 +1291,37 @@
         <v>0</v>
       </c>
       <c r="D12">
-        <f t="shared" ref="D12:D13" si="0">B12*C12</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <f t="shared" ref="E12:F13" si="0">B12*D12</f>
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <f t="shared" ref="F12:F13" si="1">C12*D12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B13">
         <v>35</v>
       </c>
       <c r="C13">
+        <v>40</v>
+      </c>
+      <c r="D13">
         <v>200</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <f t="shared" si="0"/>
         <v>7000</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="1"/>
+        <v>8000</v>
       </c>
     </row>
   </sheetData>
@@ -1287,10 +1348,10 @@
         <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="L7" t="s">
         <v>23</v>
@@ -1305,38 +1366,38 @@
         <v>19</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E10" t="s">
         <v>23</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -1358,7 +1419,7 @@
         <v>0.43999999999999995</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="L11" s="7">
         <v>-0.12</v>
@@ -1366,7 +1427,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B12">
         <v>2</v>
@@ -1388,7 +1449,7 @@
         <v>2.86</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="L12" s="7">
         <v>-0.39</v>
@@ -1396,7 +1457,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B13">
         <v>3</v>
@@ -1418,7 +1479,7 @@
         <v>0.99</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="L13" s="7">
         <v>-0.09</v>
@@ -1426,7 +1487,7 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B14">
         <v>4</v>
@@ -1448,7 +1509,7 @@
         <v>1.3199999999999998</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="L14" s="7">
         <v>-0.09</v>
@@ -1456,7 +1517,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B15">
         <v>5</v>
@@ -1478,7 +1539,7 @@
         <v>2.3833333333333333</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="L15" s="7">
         <v>-0.13</v>
@@ -1486,7 +1547,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B16">
         <v>6</v>
@@ -1508,7 +1569,7 @@
         <v>2.86</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L16" s="7">
         <v>-0.13</v>
@@ -1516,7 +1577,7 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B17">
         <v>7</v>
@@ -1538,7 +1599,7 @@
         <v>14.116666666666669</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="L17" s="7">
         <v>-0.55000000000000004</v>
@@ -1546,7 +1607,7 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B18">
         <v>8</v>
@@ -1568,7 +1629,7 @@
         <v>0.29333333333333333</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="L18" s="7">
         <v>-0.01</v>
@@ -1576,7 +1637,7 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B19">
         <v>9</v>
@@ -1598,7 +1659,7 @@
         <v>2.3100000000000005</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="L19" s="7">
         <v>-7.0000000000000007E-2</v>
@@ -1606,7 +1667,7 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B20">
         <v>10</v>
@@ -1628,7 +1689,7 @@
         <v>2.1999999999999997</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="L20" s="7">
         <v>-0.06</v>
@@ -1636,7 +1697,7 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B21">
         <v>11</v>
@@ -1658,7 +1719,7 @@
         <v>3.63</v>
       </c>
       <c r="K21" s="7" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="L21" s="7">
         <v>-0.09</v>
@@ -1666,7 +1727,7 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B22">
         <v>12</v>
@@ -1688,7 +1749,7 @@
         <v>8.3600000000000012</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="L22" s="7">
         <v>-0.19</v>
@@ -1696,7 +1757,7 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B23">
         <v>13</v>
@@ -1718,7 +1779,7 @@
         <v>6.1966666666666663</v>
       </c>
       <c r="K23" s="7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L23" s="7">
         <v>-0.13</v>
@@ -1726,7 +1787,7 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B24">
         <v>14</v>
@@ -1748,7 +1809,7 @@
         <v>2.0533333333333332</v>
       </c>
       <c r="K24" s="7" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L24" s="7">
         <v>-0.04</v>
@@ -1756,7 +1817,7 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B25">
         <v>15</v>
@@ -1778,7 +1839,7 @@
         <v>22</v>
       </c>
       <c r="K25" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="L25" s="7">
         <v>-0.4</v>
@@ -1786,7 +1847,7 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B26">
         <v>16</v>
@@ -1808,7 +1869,7 @@
         <v>5.2799999999999994</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="L26" s="7">
         <v>-0.09</v>
@@ -1816,7 +1877,7 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B27">
         <v>17</v>
@@ -1838,7 +1899,7 @@
         <v>0</v>
       </c>
       <c r="K27" s="7" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="L27" s="7">
         <v>0</v>
@@ -1846,7 +1907,7 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B28">
         <v>18</v>
@@ -1868,7 +1929,7 @@
         <v>29.04</v>
       </c>
       <c r="K28" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="L28" s="7">
         <v>-0.44</v>
@@ -1876,7 +1937,7 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B29">
         <v>19</v>
@@ -1898,7 +1959,7 @@
         <v>14.629999999999999</v>
       </c>
       <c r="K29" s="7" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="L29" s="7">
         <v>-0.21</v>
@@ -1906,7 +1967,7 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B30">
         <v>20</v>
@@ -1928,7 +1989,7 @@
         <v>15.4</v>
       </c>
       <c r="K30" s="7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="L30" s="7">
         <v>-0.21</v>
@@ -1936,7 +1997,7 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B31">
         <v>21</v>
@@ -1958,7 +2019,7 @@
         <v>0</v>
       </c>
       <c r="K31" s="7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="L31" s="7">
         <v>0</v>
@@ -1966,7 +2027,7 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B32">
         <v>22</v>
@@ -1988,7 +2049,7 @@
         <v>3.2266666666666666</v>
       </c>
       <c r="K32" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="L32" s="7">
         <v>-0.04</v>
@@ -1996,7 +2057,7 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B33">
         <v>23</v>
@@ -2018,7 +2079,7 @@
         <v>5.9033333333333333</v>
       </c>
       <c r="K33" s="7" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="L33" s="7">
         <v>-7.0000000000000007E-2</v>
@@ -2026,7 +2087,7 @@
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" s="7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B34">
         <v>24</v>
@@ -2048,7 +2109,7 @@
         <v>3.5199999999999996</v>
       </c>
       <c r="K34" s="7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="L34" s="7">
         <v>-0.04</v>
@@ -2056,7 +2117,7 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" s="7" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B35">
         <v>25</v>
@@ -2078,7 +2139,7 @@
         <v>22</v>
       </c>
       <c r="K35" s="7" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="L35" s="7">
         <v>-0.24</v>
@@ -2086,7 +2147,7 @@
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" s="7" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B36">
         <v>26</v>
@@ -2108,7 +2169,7 @@
         <v>16.206666666666667</v>
       </c>
       <c r="K36" s="7" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="L36" s="7">
         <v>-0.17</v>
@@ -2116,7 +2177,7 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B37">
         <v>27</v>
@@ -2138,7 +2199,7 @@
         <v>2.9699999999999998</v>
       </c>
       <c r="K37" s="7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="L37" s="7">
         <v>-0.03</v>
@@ -2146,7 +2207,7 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B38">
         <v>28</v>
@@ -2168,7 +2229,7 @@
         <v>2.0533333333333332</v>
       </c>
       <c r="K38" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="L38" s="7">
         <v>-0.02</v>
@@ -2176,7 +2237,7 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" s="7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B39">
         <v>29</v>
@@ -2198,7 +2259,7 @@
         <v>45.723333333333336</v>
       </c>
       <c r="K39" s="7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="L39" s="7">
         <v>-0.43</v>
@@ -2206,7 +2267,7 @@
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B40">
         <v>30</v>
@@ -2228,7 +2289,7 @@
         <v>15.4</v>
       </c>
       <c r="K40" s="7" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="L40" s="7">
         <v>-0.14000000000000001</v>
@@ -2236,7 +2297,7 @@
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" s="7" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B41">
         <v>31</v>
@@ -2258,7 +2319,7 @@
         <v>0</v>
       </c>
       <c r="K41" s="7" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="L41" s="7">
         <v>0</v>
@@ -2266,7 +2327,7 @@
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B42">
         <v>32</v>
@@ -2288,7 +2349,7 @@
         <v>14.079999999999998</v>
       </c>
       <c r="K42" s="7" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="L42" s="7">
         <v>-0.12</v>
@@ -2296,7 +2357,7 @@
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" s="7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B43">
         <v>33</v>
@@ -2318,7 +2379,7 @@
         <v>15.729999999999999</v>
       </c>
       <c r="K43" s="7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="L43" s="7">
         <v>-0.13</v>
@@ -2326,7 +2387,7 @@
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44" s="7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B44">
         <v>34</v>
@@ -2348,7 +2409,7 @@
         <v>19.946666666666669</v>
       </c>
       <c r="K44" s="7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="L44" s="7">
         <v>-0.16</v>
@@ -2356,7 +2417,7 @@
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A45" s="7" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B45">
         <v>35</v>
@@ -2378,7 +2439,7 @@
         <v>11.549999999999999</v>
       </c>
       <c r="K45" s="7" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="L45" s="7">
         <v>-0.09</v>
@@ -2386,7 +2447,7 @@
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46" s="7" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B46">
         <v>36</v>
@@ -2408,7 +2469,7 @@
         <v>0</v>
       </c>
       <c r="K46" s="7" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="L46" s="7">
         <v>0</v>
@@ -2416,7 +2477,7 @@
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A47" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B47">
         <v>37</v>
@@ -2438,7 +2499,7 @@
         <v>5.4266666666666667</v>
       </c>
       <c r="K47" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="L47" s="7">
         <v>-0.04</v>
@@ -2446,7 +2507,7 @@
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48" s="7" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B48">
         <v>38</v>
@@ -2468,7 +2529,7 @@
         <v>4.18</v>
       </c>
       <c r="K48" s="7" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="L48" s="7">
         <v>-0.03</v>
@@ -2476,7 +2537,7 @@
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B49">
         <v>39</v>
@@ -2498,7 +2559,7 @@
         <v>20.020000000000003</v>
       </c>
       <c r="K49" s="7" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="L49" s="7">
         <v>-0.14000000000000001</v>
@@ -2506,7 +2567,7 @@
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A50" s="7" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B50">
         <v>40</v>
@@ -2528,7 +2589,7 @@
         <v>45.466666666666669</v>
       </c>
       <c r="K50" s="7" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L50" s="7">
         <v>-0.31</v>
@@ -2536,7 +2597,7 @@
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B51">
         <v>41</v>
@@ -2558,7 +2619,7 @@
         <v>34.576666666666661</v>
       </c>
       <c r="K51" s="7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="L51" s="7">
         <v>-0.23</v>
@@ -2566,7 +2627,7 @@
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A52" s="7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B52">
         <v>42</v>
@@ -2588,7 +2649,7 @@
         <v>26.18</v>
       </c>
       <c r="K52" s="7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L52" s="7">
         <v>-0.17</v>
@@ -2596,7 +2657,7 @@
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B53">
         <v>43</v>
@@ -2618,7 +2679,7 @@
         <v>26.803333333333335</v>
       </c>
       <c r="K53" s="7" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="L53" s="7">
         <v>-0.17</v>
@@ -2626,7 +2687,7 @@
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A54" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B54">
         <v>44</v>
@@ -2648,7 +2709,7 @@
         <v>12.906666666666666</v>
       </c>
       <c r="K54" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="L54" s="7">
         <v>-0.08</v>
@@ -2656,7 +2717,7 @@
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B55">
         <v>45</v>
@@ -2678,7 +2739,7 @@
         <v>18.149999999999999</v>
       </c>
       <c r="K55" s="7" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="L55" s="7">
         <v>-0.11</v>
@@ -2686,7 +2747,7 @@
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A56" s="7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B56">
         <v>46</v>
@@ -2708,7 +2769,7 @@
         <v>0</v>
       </c>
       <c r="K56" s="7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="L56" s="7">
         <v>0</v>
@@ -2716,7 +2777,7 @@
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A57" s="7" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B57">
         <v>47</v>
@@ -2738,7 +2799,7 @@
         <v>3.4466666666666668</v>
       </c>
       <c r="K57" s="7" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="L57" s="7">
         <v>-0.02</v>
@@ -2746,7 +2807,7 @@
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B58">
         <v>48</v>
@@ -2768,7 +2829,7 @@
         <v>14.079999999999998</v>
       </c>
       <c r="K58" s="7" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="L58" s="7">
         <v>-0.08</v>
@@ -2776,7 +2837,7 @@
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A59" s="7" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B59">
         <v>49</v>
@@ -2798,7 +2859,7 @@
         <v>10.78</v>
       </c>
       <c r="K59" s="7" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="L59" s="7">
         <v>-0.06</v>
@@ -2806,7 +2867,7 @@
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A60" s="7" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B60">
         <v>50</v>
@@ -2828,7 +2889,7 @@
         <v>22</v>
       </c>
       <c r="K60" s="7" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="L60" s="7">
         <v>-0.12</v>
@@ -2836,7 +2897,7 @@
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A61" s="7" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B61">
         <v>51</v>
@@ -2858,7 +2919,7 @@
         <v>13.09</v>
       </c>
       <c r="K61" s="7" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="L61" s="7">
         <v>-7.0000000000000007E-2</v>
@@ -2866,7 +2927,7 @@
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62" s="7" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B62">
         <v>52</v>
@@ -2888,7 +2949,7 @@
         <v>24.786666666666665</v>
       </c>
       <c r="K62" s="7" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="L62" s="7">
         <v>-0.13</v>
@@ -2896,7 +2957,7 @@
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B63">
         <v>53</v>
@@ -2918,7 +2979,7 @@
         <v>0</v>
       </c>
       <c r="K63" s="7" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="L63" s="7">
         <v>0</v>
@@ -2926,7 +2987,7 @@
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" s="7" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B64">
         <v>54</v>
@@ -2948,7 +3009,7 @@
         <v>47.519999999999996</v>
       </c>
       <c r="K64" s="7" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="L64" s="7">
         <v>-0.24</v>
@@ -2956,7 +3017,7 @@
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A65" s="7" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B65">
         <v>55</v>
@@ -2978,7 +3039,7 @@
         <v>64.533333333333331</v>
       </c>
       <c r="K65" s="7" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="L65" s="7">
         <v>-0.32</v>
@@ -2986,7 +3047,7 @@
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A66" s="7" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B66">
         <v>56</v>
@@ -3008,7 +3069,7 @@
         <v>0</v>
       </c>
       <c r="K66" s="7" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="L66" s="7">
         <v>0</v>
@@ -3016,7 +3077,7 @@
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B67">
         <v>57</v>
@@ -3038,7 +3099,7 @@
         <v>0</v>
       </c>
       <c r="K67" s="7" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="L67" s="7">
         <v>0</v>
@@ -3046,7 +3107,7 @@
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A68" s="7" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B68">
         <v>58</v>
@@ -3068,7 +3129,7 @@
         <v>21.266666666666669</v>
       </c>
       <c r="K68" s="7" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="L68" s="7">
         <v>-0.1</v>
@@ -3076,7 +3137,7 @@
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A69" s="7" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B69">
         <v>59</v>
@@ -3098,7 +3159,7 @@
         <v>71.39</v>
       </c>
       <c r="K69" s="7" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="L69" s="7">
         <v>-0.33</v>
@@ -3106,7 +3167,7 @@
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A70" s="7" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B70">
         <v>60</v>
@@ -3128,7 +3189,7 @@
         <v>0</v>
       </c>
       <c r="K70" s="7" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="L70" s="7">
         <v>0</v>
@@ -3136,7 +3197,7 @@
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A71" s="7" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B71">
         <v>61</v>
@@ -3158,7 +3219,7 @@
         <v>11.183333333333334</v>
       </c>
       <c r="K71" s="7" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="L71" s="7">
         <v>-0.05</v>
@@ -3166,7 +3227,7 @@
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A72" s="7" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B72">
         <v>62</v>
@@ -3188,7 +3249,7 @@
         <v>59.106666666666669</v>
       </c>
       <c r="K72" s="7" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="L72" s="7">
         <v>-0.26</v>
@@ -3196,7 +3257,7 @@
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A73" s="7" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B73">
         <v>63</v>
@@ -3218,7 +3279,7 @@
         <v>60.059999999999995</v>
       </c>
       <c r="K73" s="7" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="L73" s="7">
         <v>-0.26</v>
@@ -3226,7 +3287,7 @@
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A74" s="7" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B74">
         <v>64</v>
@@ -3248,7 +3309,7 @@
         <v>7.0399999999999991</v>
       </c>
       <c r="K74" s="7" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="L74" s="7">
         <v>-0.03</v>
@@ -3256,7 +3317,7 @@
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A75" s="7" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B75">
         <v>65</v>
@@ -3278,7 +3339,7 @@
         <v>88.183333333333337</v>
       </c>
       <c r="K75" s="7" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="L75" s="7">
         <v>-0.37</v>
@@ -3286,7 +3347,7 @@
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B76">
         <v>66</v>
@@ -3308,7 +3369,7 @@
         <v>2.42</v>
       </c>
       <c r="K76" s="7" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="L76" s="7">
         <v>-0.01</v>
@@ -3316,7 +3377,7 @@
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A77" s="7" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B77">
         <v>67</v>
@@ -3338,7 +3399,7 @@
         <v>7.3699999999999992</v>
       </c>
       <c r="K77" s="7" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="L77" s="7">
         <v>-0.03</v>
@@ -3346,7 +3407,7 @@
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A78" s="7" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B78">
         <v>68</v>
@@ -3368,7 +3429,7 @@
         <v>24.933333333333334</v>
       </c>
       <c r="K78" s="7" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="L78" s="7">
         <v>-0.1</v>
@@ -3376,7 +3437,7 @@
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A79" s="7" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B79">
         <v>69</v>
@@ -3398,7 +3459,7 @@
         <v>63.25</v>
       </c>
       <c r="K79" s="7" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="L79" s="7">
         <v>-0.25</v>
@@ -3406,7 +3467,7 @@
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A80" s="7" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B80">
         <v>70</v>
@@ -3428,7 +3489,7 @@
         <v>69.300000000000011</v>
       </c>
       <c r="K80" s="7" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="L80" s="7">
         <v>-0.27</v>
@@ -3436,7 +3497,7 @@
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A81" s="7" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B81">
         <v>71</v>
@@ -3458,7 +3519,7 @@
         <v>46.859999999999992</v>
       </c>
       <c r="K81" s="7" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="L81" s="7">
         <v>-0.18</v>
@@ -3466,7 +3527,7 @@
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A82" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B82">
         <v>72</v>
@@ -3488,7 +3549,7 @@
         <v>31.68</v>
       </c>
       <c r="K82" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="L82" s="7">
         <v>-0.12</v>
@@ -3496,7 +3557,7 @@
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A83" s="7" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B83">
         <v>73</v>
@@ -3518,7 +3579,7 @@
         <v>58.886666666666656</v>
       </c>
       <c r="K83" s="7" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="L83" s="7">
         <v>-0.22</v>
@@ -3526,7 +3587,7 @@
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A84" s="7" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B84">
         <v>74</v>
@@ -3548,7 +3609,7 @@
         <v>54.266666666666666</v>
       </c>
       <c r="K84" s="7" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="L84" s="7">
         <v>-0.2</v>
@@ -3556,7 +3617,7 @@
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B85">
         <v>75</v>
@@ -3578,7 +3639,7 @@
         <v>49.5</v>
       </c>
       <c r="K85" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="L85" s="7">
         <v>-0.18</v>
@@ -3586,7 +3647,7 @@
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A86" s="7" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B86">
         <v>76</v>
@@ -3608,7 +3669,7 @@
         <v>111.46666666666667</v>
       </c>
       <c r="K86" s="7" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="L86" s="7">
         <v>-0.4</v>
@@ -3616,7 +3677,7 @@
     </row>
     <row r="87" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A87" s="7" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B87">
         <v>77</v>
@@ -3638,7 +3699,7 @@
         <v>59.289999999999992</v>
       </c>
       <c r="K87" s="7" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="L87" s="7">
         <v>-0.21</v>
@@ -3646,7 +3707,7 @@
     </row>
     <row r="88" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A88" s="7" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B88">
         <v>78</v>
@@ -3668,7 +3729,7 @@
         <v>111.54</v>
       </c>
       <c r="K88" s="7" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="L88" s="7">
         <v>-0.39</v>
@@ -3676,7 +3737,7 @@
     </row>
     <row r="89" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A89" s="7" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B89">
         <v>79</v>
@@ -3698,7 +3759,7 @@
         <v>199.86999999999998</v>
       </c>
       <c r="K89" s="7" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="L89" s="7">
         <v>-0.69</v>
@@ -3706,7 +3767,7 @@
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A90" s="7" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B90">
         <v>80</v>
@@ -3728,7 +3789,7 @@
         <v>0</v>
       </c>
       <c r="K90" s="7" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="L90" s="7">
         <v>0</v>
@@ -3736,7 +3797,7 @@
     </row>
     <row r="91" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A91" s="7" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B91">
         <v>81</v>
@@ -3758,7 +3819,7 @@
         <v>20.790000000000003</v>
       </c>
       <c r="K91" s="7" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="L91" s="7">
         <v>-7.0000000000000007E-2</v>
@@ -3766,7 +3827,7 @@
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A92" s="7" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B92">
         <v>82</v>
@@ -3788,7 +3849,7 @@
         <v>171.37999999999997</v>
       </c>
       <c r="K92" s="7" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="L92" s="7">
         <v>-0.56999999999999995</v>
@@ -3796,7 +3857,7 @@
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A93" s="7" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B93">
         <v>83</v>
@@ -3818,7 +3879,7 @@
         <v>203.90333333333334</v>
       </c>
       <c r="K93" s="7" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="L93" s="7">
         <v>-0.67</v>
@@ -3826,7 +3887,7 @@
     </row>
     <row r="94" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A94" s="7" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B94">
         <v>84</v>
@@ -3848,7 +3909,7 @@
         <v>15.4</v>
       </c>
       <c r="K94" s="7" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="L94" s="7">
         <v>-0.05</v>
@@ -3866,7 +3927,7 @@
   <sheetData>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -3894,21 +3955,21 @@
         <v>24</v>
       </c>
       <c r="D8" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C10" t="s">
         <v>23</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
chore: fix spreadsheet that got overwritten in merge
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/16-lulucf/16.1-lulucf.xlsx
+++ b/packages/calculators/src/modules/test/16-lulucf/16.1-lulucf.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/16-lulucf/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{467B2523-29EF-0742-9B74-29AC65CA6F22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB847984-2549-C142-8149-702321047583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51200" yWindow="13240" windowWidth="28800" windowHeight="27420" activeTab="3" xr2:uid="{CC0FEAF9-C40F-694B-BCB9-117AFB86C05D}"/>
+    <workbookView xWindow="51200" yWindow="13240" windowWidth="28800" windowHeight="27420" activeTab="1" xr2:uid="{CC0FEAF9-C40F-694B-BCB9-117AFB86C05D}"/>
   </bookViews>
   <sheets>
     <sheet name="16.1.1.2" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="139">
   <si>
     <t>Scenario</t>
   </si>
@@ -152,22 +152,13 @@
     <t>Deforesting</t>
   </si>
   <si>
-    <t>Egijy</t>
-  </si>
-  <si>
     <t>agijy</t>
   </si>
   <si>
-    <t>ELUCgjy</t>
-  </si>
-  <si>
     <t>Emissions from biomass burning</t>
   </si>
   <si>
     <t>t CO2e</t>
-  </si>
-  <si>
-    <t>t CO2e / ha</t>
   </si>
   <si>
     <t>Area burnt</t>
@@ -518,6 +509,30 @@
   </si>
   <si>
     <t>Yalgoo</t>
+  </si>
+  <si>
+    <t>Eg=ch4,I,j,y</t>
+  </si>
+  <si>
+    <t>t CH4 / ha</t>
+  </si>
+  <si>
+    <t>t N2O / ha</t>
+  </si>
+  <si>
+    <t>Eg=n2o,I,j,y</t>
+  </si>
+  <si>
+    <t>ELUCg=ch4jy</t>
+  </si>
+  <si>
+    <t>t CH4</t>
+  </si>
+  <si>
+    <t>t N2O</t>
+  </si>
+  <si>
+    <t>ELUCg=n2ojy</t>
   </si>
 </sst>
 </file>
@@ -946,16 +961,16 @@
   <sheetData>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -1161,64 +1176,89 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92CDB52C-734F-7046-ACDC-C5573D991542}">
-  <dimension ref="A4:D13"/>
+  <dimension ref="A4:F13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="16.1640625" customWidth="1"/>
-    <col min="3" max="3" width="18.1640625" customWidth="1"/>
-    <col min="4" max="4" width="19.33203125" customWidth="1"/>
+    <col min="2" max="3" width="16.1640625" customWidth="1"/>
+    <col min="4" max="4" width="18.1640625" customWidth="1"/>
+    <col min="5" max="5" width="19.33203125" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+      <c r="C4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>5</v>
       </c>
       <c r="C6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>31</v>
+        <v>132</v>
       </c>
       <c r="C7" t="s">
+        <v>133</v>
+      </c>
+      <c r="D7" t="s">
         <v>24</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
+        <v>136</v>
+      </c>
+      <c r="F7" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="B9" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B9" s="1" t="s">
-        <v>33</v>
-      </c>
       <c r="C9" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>0</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E10" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -1226,16 +1266,23 @@
         <v>25</v>
       </c>
       <c r="C11">
+        <v>4</v>
+      </c>
+      <c r="D11">
         <v>5</v>
       </c>
-      <c r="D11">
-        <f>B11*C11</f>
+      <c r="E11">
+        <f>B11*D11</f>
         <v>125</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="F11">
+        <f>C11*D11</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -1244,23 +1291,37 @@
         <v>0</v>
       </c>
       <c r="D12">
-        <f t="shared" ref="D12:D13" si="0">B12*C12</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <f t="shared" ref="E12:F13" si="0">B12*D12</f>
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <f t="shared" ref="F12:F13" si="1">C12*D12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B13">
         <v>35</v>
       </c>
       <c r="C13">
+        <v>40</v>
+      </c>
+      <c r="D13">
         <v>200</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <f t="shared" si="0"/>
         <v>7000</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="1"/>
+        <v>8000</v>
       </c>
     </row>
   </sheetData>
@@ -1287,10 +1348,10 @@
         <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="L7" t="s">
         <v>23</v>
@@ -1305,38 +1366,38 @@
         <v>19</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E10" t="s">
         <v>23</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -1358,7 +1419,7 @@
         <v>0.43999999999999995</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="L11" s="7">
         <v>-0.12</v>
@@ -1366,7 +1427,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B12">
         <v>2</v>
@@ -1388,7 +1449,7 @@
         <v>2.86</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="L12" s="7">
         <v>-0.39</v>
@@ -1396,7 +1457,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B13">
         <v>3</v>
@@ -1418,7 +1479,7 @@
         <v>0.99</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="L13" s="7">
         <v>-0.09</v>
@@ -1426,7 +1487,7 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B14">
         <v>4</v>
@@ -1448,7 +1509,7 @@
         <v>1.3199999999999998</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="L14" s="7">
         <v>-0.09</v>
@@ -1456,7 +1517,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B15">
         <v>5</v>
@@ -1478,7 +1539,7 @@
         <v>2.3833333333333333</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="L15" s="7">
         <v>-0.13</v>
@@ -1486,7 +1547,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B16">
         <v>6</v>
@@ -1508,7 +1569,7 @@
         <v>2.86</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L16" s="7">
         <v>-0.13</v>
@@ -1516,7 +1577,7 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B17">
         <v>7</v>
@@ -1538,7 +1599,7 @@
         <v>14.116666666666669</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="L17" s="7">
         <v>-0.55000000000000004</v>
@@ -1546,7 +1607,7 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B18">
         <v>8</v>
@@ -1568,7 +1629,7 @@
         <v>0.29333333333333333</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="L18" s="7">
         <v>-0.01</v>
@@ -1576,7 +1637,7 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B19">
         <v>9</v>
@@ -1598,7 +1659,7 @@
         <v>2.3100000000000005</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="L19" s="7">
         <v>-7.0000000000000007E-2</v>
@@ -1606,7 +1667,7 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B20">
         <v>10</v>
@@ -1628,7 +1689,7 @@
         <v>2.1999999999999997</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="L20" s="7">
         <v>-0.06</v>
@@ -1636,7 +1697,7 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B21">
         <v>11</v>
@@ -1658,7 +1719,7 @@
         <v>3.63</v>
       </c>
       <c r="K21" s="7" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="L21" s="7">
         <v>-0.09</v>
@@ -1666,7 +1727,7 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B22">
         <v>12</v>
@@ -1688,7 +1749,7 @@
         <v>8.3600000000000012</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="L22" s="7">
         <v>-0.19</v>
@@ -1696,7 +1757,7 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B23">
         <v>13</v>
@@ -1718,7 +1779,7 @@
         <v>6.1966666666666663</v>
       </c>
       <c r="K23" s="7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L23" s="7">
         <v>-0.13</v>
@@ -1726,7 +1787,7 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B24">
         <v>14</v>
@@ -1748,7 +1809,7 @@
         <v>2.0533333333333332</v>
       </c>
       <c r="K24" s="7" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L24" s="7">
         <v>-0.04</v>
@@ -1756,7 +1817,7 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B25">
         <v>15</v>
@@ -1778,7 +1839,7 @@
         <v>22</v>
       </c>
       <c r="K25" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="L25" s="7">
         <v>-0.4</v>
@@ -1786,7 +1847,7 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B26">
         <v>16</v>
@@ -1808,7 +1869,7 @@
         <v>5.2799999999999994</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="L26" s="7">
         <v>-0.09</v>
@@ -1816,7 +1877,7 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B27">
         <v>17</v>
@@ -1838,7 +1899,7 @@
         <v>0</v>
       </c>
       <c r="K27" s="7" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="L27" s="7">
         <v>0</v>
@@ -1846,7 +1907,7 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B28">
         <v>18</v>
@@ -1868,7 +1929,7 @@
         <v>29.04</v>
       </c>
       <c r="K28" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="L28" s="7">
         <v>-0.44</v>
@@ -1876,7 +1937,7 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B29">
         <v>19</v>
@@ -1898,7 +1959,7 @@
         <v>14.629999999999999</v>
       </c>
       <c r="K29" s="7" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="L29" s="7">
         <v>-0.21</v>
@@ -1906,7 +1967,7 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B30">
         <v>20</v>
@@ -1928,7 +1989,7 @@
         <v>15.4</v>
       </c>
       <c r="K30" s="7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="L30" s="7">
         <v>-0.21</v>
@@ -1936,7 +1997,7 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B31">
         <v>21</v>
@@ -1958,7 +2019,7 @@
         <v>0</v>
       </c>
       <c r="K31" s="7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="L31" s="7">
         <v>0</v>
@@ -1966,7 +2027,7 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B32">
         <v>22</v>
@@ -1988,7 +2049,7 @@
         <v>3.2266666666666666</v>
       </c>
       <c r="K32" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="L32" s="7">
         <v>-0.04</v>
@@ -1996,7 +2057,7 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B33">
         <v>23</v>
@@ -2018,7 +2079,7 @@
         <v>5.9033333333333333</v>
       </c>
       <c r="K33" s="7" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="L33" s="7">
         <v>-7.0000000000000007E-2</v>
@@ -2026,7 +2087,7 @@
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" s="7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B34">
         <v>24</v>
@@ -2048,7 +2109,7 @@
         <v>3.5199999999999996</v>
       </c>
       <c r="K34" s="7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="L34" s="7">
         <v>-0.04</v>
@@ -2056,7 +2117,7 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" s="7" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B35">
         <v>25</v>
@@ -2078,7 +2139,7 @@
         <v>22</v>
       </c>
       <c r="K35" s="7" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="L35" s="7">
         <v>-0.24</v>
@@ -2086,7 +2147,7 @@
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" s="7" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B36">
         <v>26</v>
@@ -2108,7 +2169,7 @@
         <v>16.206666666666667</v>
       </c>
       <c r="K36" s="7" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="L36" s="7">
         <v>-0.17</v>
@@ -2116,7 +2177,7 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B37">
         <v>27</v>
@@ -2138,7 +2199,7 @@
         <v>2.9699999999999998</v>
       </c>
       <c r="K37" s="7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="L37" s="7">
         <v>-0.03</v>
@@ -2146,7 +2207,7 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B38">
         <v>28</v>
@@ -2168,7 +2229,7 @@
         <v>2.0533333333333332</v>
       </c>
       <c r="K38" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="L38" s="7">
         <v>-0.02</v>
@@ -2176,7 +2237,7 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" s="7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B39">
         <v>29</v>
@@ -2198,7 +2259,7 @@
         <v>45.723333333333336</v>
       </c>
       <c r="K39" s="7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="L39" s="7">
         <v>-0.43</v>
@@ -2206,7 +2267,7 @@
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B40">
         <v>30</v>
@@ -2228,7 +2289,7 @@
         <v>15.4</v>
       </c>
       <c r="K40" s="7" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="L40" s="7">
         <v>-0.14000000000000001</v>
@@ -2236,7 +2297,7 @@
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" s="7" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B41">
         <v>31</v>
@@ -2258,7 +2319,7 @@
         <v>0</v>
       </c>
       <c r="K41" s="7" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="L41" s="7">
         <v>0</v>
@@ -2266,7 +2327,7 @@
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B42">
         <v>32</v>
@@ -2288,7 +2349,7 @@
         <v>14.079999999999998</v>
       </c>
       <c r="K42" s="7" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="L42" s="7">
         <v>-0.12</v>
@@ -2296,7 +2357,7 @@
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" s="7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B43">
         <v>33</v>
@@ -2318,7 +2379,7 @@
         <v>15.729999999999999</v>
       </c>
       <c r="K43" s="7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="L43" s="7">
         <v>-0.13</v>
@@ -2326,7 +2387,7 @@
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44" s="7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B44">
         <v>34</v>
@@ -2348,7 +2409,7 @@
         <v>19.946666666666669</v>
       </c>
       <c r="K44" s="7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="L44" s="7">
         <v>-0.16</v>
@@ -2356,7 +2417,7 @@
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A45" s="7" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B45">
         <v>35</v>
@@ -2378,7 +2439,7 @@
         <v>11.549999999999999</v>
       </c>
       <c r="K45" s="7" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="L45" s="7">
         <v>-0.09</v>
@@ -2386,7 +2447,7 @@
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46" s="7" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B46">
         <v>36</v>
@@ -2408,7 +2469,7 @@
         <v>0</v>
       </c>
       <c r="K46" s="7" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="L46" s="7">
         <v>0</v>
@@ -2416,7 +2477,7 @@
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A47" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B47">
         <v>37</v>
@@ -2438,7 +2499,7 @@
         <v>5.4266666666666667</v>
       </c>
       <c r="K47" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="L47" s="7">
         <v>-0.04</v>
@@ -2446,7 +2507,7 @@
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48" s="7" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B48">
         <v>38</v>
@@ -2468,7 +2529,7 @@
         <v>4.18</v>
       </c>
       <c r="K48" s="7" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="L48" s="7">
         <v>-0.03</v>
@@ -2476,7 +2537,7 @@
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B49">
         <v>39</v>
@@ -2498,7 +2559,7 @@
         <v>20.020000000000003</v>
       </c>
       <c r="K49" s="7" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="L49" s="7">
         <v>-0.14000000000000001</v>
@@ -2506,7 +2567,7 @@
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A50" s="7" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B50">
         <v>40</v>
@@ -2528,7 +2589,7 @@
         <v>45.466666666666669</v>
       </c>
       <c r="K50" s="7" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L50" s="7">
         <v>-0.31</v>
@@ -2536,7 +2597,7 @@
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B51">
         <v>41</v>
@@ -2558,7 +2619,7 @@
         <v>34.576666666666661</v>
       </c>
       <c r="K51" s="7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="L51" s="7">
         <v>-0.23</v>
@@ -2566,7 +2627,7 @@
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A52" s="7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B52">
         <v>42</v>
@@ -2588,7 +2649,7 @@
         <v>26.18</v>
       </c>
       <c r="K52" s="7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L52" s="7">
         <v>-0.17</v>
@@ -2596,7 +2657,7 @@
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B53">
         <v>43</v>
@@ -2618,7 +2679,7 @@
         <v>26.803333333333335</v>
       </c>
       <c r="K53" s="7" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="L53" s="7">
         <v>-0.17</v>
@@ -2626,7 +2687,7 @@
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A54" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B54">
         <v>44</v>
@@ -2648,7 +2709,7 @@
         <v>12.906666666666666</v>
       </c>
       <c r="K54" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="L54" s="7">
         <v>-0.08</v>
@@ -2656,7 +2717,7 @@
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B55">
         <v>45</v>
@@ -2678,7 +2739,7 @@
         <v>18.149999999999999</v>
       </c>
       <c r="K55" s="7" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="L55" s="7">
         <v>-0.11</v>
@@ -2686,7 +2747,7 @@
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A56" s="7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B56">
         <v>46</v>
@@ -2708,7 +2769,7 @@
         <v>0</v>
       </c>
       <c r="K56" s="7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="L56" s="7">
         <v>0</v>
@@ -2716,7 +2777,7 @@
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A57" s="7" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B57">
         <v>47</v>
@@ -2738,7 +2799,7 @@
         <v>3.4466666666666668</v>
       </c>
       <c r="K57" s="7" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="L57" s="7">
         <v>-0.02</v>
@@ -2746,7 +2807,7 @@
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B58">
         <v>48</v>
@@ -2768,7 +2829,7 @@
         <v>14.079999999999998</v>
       </c>
       <c r="K58" s="7" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="L58" s="7">
         <v>-0.08</v>
@@ -2776,7 +2837,7 @@
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A59" s="7" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B59">
         <v>49</v>
@@ -2798,7 +2859,7 @@
         <v>10.78</v>
       </c>
       <c r="K59" s="7" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="L59" s="7">
         <v>-0.06</v>
@@ -2806,7 +2867,7 @@
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A60" s="7" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B60">
         <v>50</v>
@@ -2828,7 +2889,7 @@
         <v>22</v>
       </c>
       <c r="K60" s="7" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="L60" s="7">
         <v>-0.12</v>
@@ -2836,7 +2897,7 @@
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A61" s="7" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B61">
         <v>51</v>
@@ -2858,7 +2919,7 @@
         <v>13.09</v>
       </c>
       <c r="K61" s="7" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="L61" s="7">
         <v>-7.0000000000000007E-2</v>
@@ -2866,7 +2927,7 @@
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62" s="7" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B62">
         <v>52</v>
@@ -2888,7 +2949,7 @@
         <v>24.786666666666665</v>
       </c>
       <c r="K62" s="7" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="L62" s="7">
         <v>-0.13</v>
@@ -2896,7 +2957,7 @@
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B63">
         <v>53</v>
@@ -2918,7 +2979,7 @@
         <v>0</v>
       </c>
       <c r="K63" s="7" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="L63" s="7">
         <v>0</v>
@@ -2926,7 +2987,7 @@
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" s="7" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B64">
         <v>54</v>
@@ -2948,7 +3009,7 @@
         <v>47.519999999999996</v>
       </c>
       <c r="K64" s="7" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="L64" s="7">
         <v>-0.24</v>
@@ -2956,7 +3017,7 @@
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A65" s="7" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B65">
         <v>55</v>
@@ -2978,7 +3039,7 @@
         <v>64.533333333333331</v>
       </c>
       <c r="K65" s="7" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="L65" s="7">
         <v>-0.32</v>
@@ -2986,7 +3047,7 @@
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A66" s="7" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B66">
         <v>56</v>
@@ -3008,7 +3069,7 @@
         <v>0</v>
       </c>
       <c r="K66" s="7" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="L66" s="7">
         <v>0</v>
@@ -3016,7 +3077,7 @@
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B67">
         <v>57</v>
@@ -3038,7 +3099,7 @@
         <v>0</v>
       </c>
       <c r="K67" s="7" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="L67" s="7">
         <v>0</v>
@@ -3046,7 +3107,7 @@
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A68" s="7" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B68">
         <v>58</v>
@@ -3068,7 +3129,7 @@
         <v>21.266666666666669</v>
       </c>
       <c r="K68" s="7" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="L68" s="7">
         <v>-0.1</v>
@@ -3076,7 +3137,7 @@
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A69" s="7" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B69">
         <v>59</v>
@@ -3098,7 +3159,7 @@
         <v>71.39</v>
       </c>
       <c r="K69" s="7" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="L69" s="7">
         <v>-0.33</v>
@@ -3106,7 +3167,7 @@
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A70" s="7" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B70">
         <v>60</v>
@@ -3128,7 +3189,7 @@
         <v>0</v>
       </c>
       <c r="K70" s="7" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="L70" s="7">
         <v>0</v>
@@ -3136,7 +3197,7 @@
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A71" s="7" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B71">
         <v>61</v>
@@ -3158,7 +3219,7 @@
         <v>11.183333333333334</v>
       </c>
       <c r="K71" s="7" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="L71" s="7">
         <v>-0.05</v>
@@ -3166,7 +3227,7 @@
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A72" s="7" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B72">
         <v>62</v>
@@ -3188,7 +3249,7 @@
         <v>59.106666666666669</v>
       </c>
       <c r="K72" s="7" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="L72" s="7">
         <v>-0.26</v>
@@ -3196,7 +3257,7 @@
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A73" s="7" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B73">
         <v>63</v>
@@ -3218,7 +3279,7 @@
         <v>60.059999999999995</v>
       </c>
       <c r="K73" s="7" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="L73" s="7">
         <v>-0.26</v>
@@ -3226,7 +3287,7 @@
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A74" s="7" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B74">
         <v>64</v>
@@ -3248,7 +3309,7 @@
         <v>7.0399999999999991</v>
       </c>
       <c r="K74" s="7" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="L74" s="7">
         <v>-0.03</v>
@@ -3256,7 +3317,7 @@
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A75" s="7" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B75">
         <v>65</v>
@@ -3278,7 +3339,7 @@
         <v>88.183333333333337</v>
       </c>
       <c r="K75" s="7" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="L75" s="7">
         <v>-0.37</v>
@@ -3286,7 +3347,7 @@
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B76">
         <v>66</v>
@@ -3308,7 +3369,7 @@
         <v>2.42</v>
       </c>
       <c r="K76" s="7" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="L76" s="7">
         <v>-0.01</v>
@@ -3316,7 +3377,7 @@
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A77" s="7" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B77">
         <v>67</v>
@@ -3338,7 +3399,7 @@
         <v>7.3699999999999992</v>
       </c>
       <c r="K77" s="7" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="L77" s="7">
         <v>-0.03</v>
@@ -3346,7 +3407,7 @@
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A78" s="7" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B78">
         <v>68</v>
@@ -3368,7 +3429,7 @@
         <v>24.933333333333334</v>
       </c>
       <c r="K78" s="7" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="L78" s="7">
         <v>-0.1</v>
@@ -3376,7 +3437,7 @@
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A79" s="7" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B79">
         <v>69</v>
@@ -3398,7 +3459,7 @@
         <v>63.25</v>
       </c>
       <c r="K79" s="7" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="L79" s="7">
         <v>-0.25</v>
@@ -3406,7 +3467,7 @@
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A80" s="7" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B80">
         <v>70</v>
@@ -3428,7 +3489,7 @@
         <v>69.300000000000011</v>
       </c>
       <c r="K80" s="7" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="L80" s="7">
         <v>-0.27</v>
@@ -3436,7 +3497,7 @@
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A81" s="7" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B81">
         <v>71</v>
@@ -3458,7 +3519,7 @@
         <v>46.859999999999992</v>
       </c>
       <c r="K81" s="7" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="L81" s="7">
         <v>-0.18</v>
@@ -3466,7 +3527,7 @@
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A82" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B82">
         <v>72</v>
@@ -3488,7 +3549,7 @@
         <v>31.68</v>
       </c>
       <c r="K82" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="L82" s="7">
         <v>-0.12</v>
@@ -3496,7 +3557,7 @@
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A83" s="7" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B83">
         <v>73</v>
@@ -3518,7 +3579,7 @@
         <v>58.886666666666656</v>
       </c>
       <c r="K83" s="7" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="L83" s="7">
         <v>-0.22</v>
@@ -3526,7 +3587,7 @@
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A84" s="7" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B84">
         <v>74</v>
@@ -3548,7 +3609,7 @@
         <v>54.266666666666666</v>
       </c>
       <c r="K84" s="7" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="L84" s="7">
         <v>-0.2</v>
@@ -3556,7 +3617,7 @@
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B85">
         <v>75</v>
@@ -3578,7 +3639,7 @@
         <v>49.5</v>
       </c>
       <c r="K85" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="L85" s="7">
         <v>-0.18</v>
@@ -3586,7 +3647,7 @@
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A86" s="7" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B86">
         <v>76</v>
@@ -3608,7 +3669,7 @@
         <v>111.46666666666667</v>
       </c>
       <c r="K86" s="7" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="L86" s="7">
         <v>-0.4</v>
@@ -3616,7 +3677,7 @@
     </row>
     <row r="87" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A87" s="7" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B87">
         <v>77</v>
@@ -3638,7 +3699,7 @@
         <v>59.289999999999992</v>
       </c>
       <c r="K87" s="7" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="L87" s="7">
         <v>-0.21</v>
@@ -3646,7 +3707,7 @@
     </row>
     <row r="88" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A88" s="7" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B88">
         <v>78</v>
@@ -3668,7 +3729,7 @@
         <v>111.54</v>
       </c>
       <c r="K88" s="7" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="L88" s="7">
         <v>-0.39</v>
@@ -3676,7 +3737,7 @@
     </row>
     <row r="89" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A89" s="7" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B89">
         <v>79</v>
@@ -3698,7 +3759,7 @@
         <v>199.86999999999998</v>
       </c>
       <c r="K89" s="7" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="L89" s="7">
         <v>-0.69</v>
@@ -3706,7 +3767,7 @@
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A90" s="7" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B90">
         <v>80</v>
@@ -3728,7 +3789,7 @@
         <v>0</v>
       </c>
       <c r="K90" s="7" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="L90" s="7">
         <v>0</v>
@@ -3736,7 +3797,7 @@
     </row>
     <row r="91" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A91" s="7" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B91">
         <v>81</v>
@@ -3758,7 +3819,7 @@
         <v>20.790000000000003</v>
       </c>
       <c r="K91" s="7" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="L91" s="7">
         <v>-7.0000000000000007E-2</v>
@@ -3766,7 +3827,7 @@
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A92" s="7" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B92">
         <v>82</v>
@@ -3788,7 +3849,7 @@
         <v>171.37999999999997</v>
       </c>
       <c r="K92" s="7" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="L92" s="7">
         <v>-0.56999999999999995</v>
@@ -3796,7 +3857,7 @@
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A93" s="7" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B93">
         <v>83</v>
@@ -3818,7 +3879,7 @@
         <v>203.90333333333334</v>
       </c>
       <c r="K93" s="7" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="L93" s="7">
         <v>-0.67</v>
@@ -3826,7 +3887,7 @@
     </row>
     <row r="94" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A94" s="7" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B94">
         <v>84</v>
@@ -3848,7 +3909,7 @@
         <v>15.4</v>
       </c>
       <c r="K94" s="7" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="L94" s="7">
         <v>-0.05</v>
@@ -3866,7 +3927,7 @@
   <sheetData>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -3894,21 +3955,21 @@
         <v>24</v>
       </c>
       <c r="D8" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C10" t="s">
         <v>23</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>